<commit_message>
feat: add comprehensive PHI compliance scanning results, expand test data, and document engine hardening enhancements.
</commit_message>
<xml_diff>
--- a/sample_data/messy_data.xlsx
+++ b/sample_data/messy_data.xlsx
@@ -8,7 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Noise" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Messy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numeric_IDs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Noise" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,7 +539,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4567 8901 2341</t>
+          <t>4567.8901.2341</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -575,7 +577,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MNOFS6789L</t>
+          <t>Mnofs6789L</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -634,74 +636,317 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>employee_id</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>notes</t>
+          <t>category</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>N001</t>
+          <t>PAN: ABCPD1234E, Mobile: 9876543210</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Order ref</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Ref: 1234567890123 (13 digits — not Aadhaar)</t>
+          <t>combo</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>N002</t>
+          <t>Aadhar No: 678901234560</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Turnover: 5000000000 (10 digit amount)</t>
+          <t>labeled</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>N003</t>
+          <t>XXXX XXXX 1234</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Timestamp</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+          <t>masked</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>**** **** 5678</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>masked_stars</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ABC PD 1234 E</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>spaced_pan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7890/1234/5674</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>slashed_aadhaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>98765.43210</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>dotted_mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>(91) 9876543210</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>parens_mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ABCPD1234E@company.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>email_fp</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>aadhaar_no</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>phone_no</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>890123456784</v>
+      </c>
+      <c r="B2" t="n">
+        <v>9876543210</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Test Person</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>901234567892</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8765432109</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Another Person</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ref: 1234567890123 (13 digits — not Aadhaar)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>order_ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Turnover: 5000000000 (10 digit amount)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>20261101120000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>₹9876543210</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>INR 8765432109</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>inr_amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rs. 7654321098</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>rs_amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>INV-9876543210</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>invoice</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ORD#8765432109</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EMP5432109876</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>emp_id</t>
         </is>
       </c>
     </row>

</xml_diff>